<commit_message>
feat: multi-persona seed system with profile.md narrative layer
- Refactor seed-data.js into thin loader + persona modules (scripts/personas/)
- Add Alex (Taiwanese, Google L7, ~$5.5M NW) and Sophia (British, Anthropic, ~$4.3M NW)
- Add profile.md narrative memory for agents/skills context
- Update tax agent, portfolio skill, onboarding skill to read profile.md
- Add /api/profile/memory endpoint and SSE watcher
- Simplify persona filenames to first name only (alex.js, sophia.js)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/angel-investment.xlsx
+++ b/data/angel-investment.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L2"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -453,10 +453,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>startup-nexaflow</v>
+        <v>startup-safeguard</v>
       </c>
       <c r="B2" t="str">
-        <v>NexaFlow</v>
+        <v>SafeGuard AI</v>
       </c>
       <c r="C2" t="str">
         <v>PRIVATE</v>
@@ -465,13 +465,13 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>50000</v>
+        <v>25000</v>
       </c>
       <c r="F2">
-        <v>120000</v>
+        <v>25000</v>
       </c>
       <c r="G2" t="str">
-        <v>Seed round. AI-powered supply chain. Est. valuation $12M. 1% equity.</v>
+        <v>Seed round. AI safety startup — alignment research commercialization. Ex-Google DeepMind founder. Invested through Anthropic colleague. Too early to mark up.</v>
       </c>
       <c r="H2" t="str">
         <v>taxable</v>
@@ -480,94 +480,18 @@
         <v>Direct Investment</v>
       </c>
       <c r="J2">
-        <v>50000</v>
+        <v>25000</v>
       </c>
       <c r="K2" t="str">
-        <v>2023-04-01</v>
+        <v>2025-08-01</v>
       </c>
       <c r="L2" t="str">
-        <v>2026-02-11</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>startup-carbonlens</v>
-      </c>
-      <c r="B3" t="str">
-        <v>CarbonLens</v>
-      </c>
-      <c r="C3" t="str">
-        <v>PRIVATE</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>75000</v>
-      </c>
-      <c r="F3">
-        <v>95000</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Series A. Carbon credit marketplace. Est. valuation $25M. 0.38% equity.</v>
-      </c>
-      <c r="H3" t="str">
-        <v>taxable</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Direct Investment</v>
-      </c>
-      <c r="J3">
-        <v>75000</v>
-      </c>
-      <c r="K3" t="str">
-        <v>2024-01-15</v>
-      </c>
-      <c r="L3" t="str">
-        <v>2026-02-11</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>startup-vaultedge</v>
-      </c>
-      <c r="B4" t="str">
-        <v>VaultEdge</v>
-      </c>
-      <c r="C4" t="str">
-        <v>PRIVATE</v>
-      </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
-      <c r="E4">
-        <v>25000</v>
-      </c>
-      <c r="F4">
-        <v>25000</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Pre-seed. Decentralized identity for fintech. Earliest stage, highest risk.</v>
-      </c>
-      <c r="H4" t="str">
-        <v>taxable</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Direct Investment</v>
-      </c>
-      <c r="J4">
-        <v>25000</v>
-      </c>
-      <c r="K4" t="str">
-        <v>2025-06-01</v>
-      </c>
-      <c r="L4" t="str">
-        <v>2026-02-11</v>
+        <v>2026-02-12</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: category-aware display profiles for dashboard tables
Each asset category now renders context-appropriate columns instead of
the same 5-column layout. Added 6 display profiles (market-traded,
cash-like, yield-bearing, private-equity, employee-equity, physical-asset)
driven by a displayProfile field in categories.json.

- Add public/js/config/display-profiles.js as single source of truth
- Refactor category-detail.js: replace renderHoldingsTable/renderEquityTable
  with unified renderProfileTable driven by profile config
- Add displayProfile to categoryMeta in both persona files
- Move VNQ (REIT ETF) from real-estate to stocks (exchange-traded)
- Add classification-rules.md reference doc with decision tree
- Update onboarding + portfolio skills to check classification rules
  before writing assets

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/angel-investment.xlsx
+++ b/data/angel-investment.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -453,10 +453,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>startup-safeguard</v>
+        <v>startup-nexaflow</v>
       </c>
       <c r="B2" t="str">
-        <v>SafeGuard AI</v>
+        <v>NexaFlow</v>
       </c>
       <c r="C2" t="str">
         <v>PRIVATE</v>
@@ -465,13 +465,13 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>25000</v>
+        <v>50000</v>
       </c>
       <c r="F2">
-        <v>25000</v>
+        <v>120000</v>
       </c>
       <c r="G2" t="str">
-        <v>Seed round. AI safety startup — alignment research commercialization. Ex-Google DeepMind founder. Invested through Anthropic colleague. Too early to mark up.</v>
+        <v>Seed round. AI-powered supply chain. Est. valuation $12M. 1% equity.</v>
       </c>
       <c r="H2" t="str">
         <v>taxable</v>
@@ -480,18 +480,56 @@
         <v>Direct Investment</v>
       </c>
       <c r="J2">
+        <v>50000</v>
+      </c>
+      <c r="K2" t="str">
+        <v>2023-04-01</v>
+      </c>
+      <c r="L2" t="str">
+        <v>2026-02-12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>startup-vaultedge</v>
+      </c>
+      <c r="B3" t="str">
+        <v>VaultEdge</v>
+      </c>
+      <c r="C3" t="str">
+        <v>PRIVATE</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
         <v>25000</v>
       </c>
-      <c r="K2" t="str">
-        <v>2025-08-01</v>
-      </c>
-      <c r="L2" t="str">
+      <c r="F3">
+        <v>25000</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Pre-seed. Decentralized identity for fintech. Earliest stage, highest risk.</v>
+      </c>
+      <c r="H3" t="str">
+        <v>taxable</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Direct Investment</v>
+      </c>
+      <c r="J3">
+        <v>25000</v>
+      </c>
+      <c r="K3" t="str">
+        <v>2025-06-01</v>
+      </c>
+      <c r="L3" t="str">
         <v>2026-02-12</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: hidden tax liability — collectible 28% rate, Section 121 exclusion, per-asset rate display
Hidden Liabilities now correctly handles:
- Collectibles (jewelry, art) at 28% LTCG rate instead of standard 20%
- Primary residence Section 121 exclusion ($500K MFJ)
- Per-asset effective rate column in the table
Also includes: write-through cache timestamps, taxable events year display,
short-term rate correction (35% → 37%), dashboard data updates.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/angel-investment.xlsx
+++ b/data/angel-investment.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -453,10 +453,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>startup-safeguard</v>
+        <v>startup-nexaflow</v>
       </c>
       <c r="B2" t="str">
-        <v>SafeGuard AI</v>
+        <v>NexaFlow</v>
       </c>
       <c r="C2" t="str">
         <v>PRIVATE</v>
@@ -465,13 +465,13 @@
         <v>1</v>
       </c>
       <c r="E2">
-        <v>25000</v>
+        <v>50000</v>
       </c>
       <c r="F2">
-        <v>25000</v>
+        <v>120000</v>
       </c>
       <c r="G2" t="str">
-        <v>Seed round. AI safety startup — alignment research commercialization. Ex-Google DeepMind founder. Invested through Anthropic colleague. Too early to mark up.</v>
+        <v>Seed round. AI-powered supply chain. Est. valuation $12M. 1% equity.</v>
       </c>
       <c r="H2" t="str">
         <v>taxable</v>
@@ -480,18 +480,56 @@
         <v>Direct Investment</v>
       </c>
       <c r="J2">
+        <v>50000</v>
+      </c>
+      <c r="K2" t="str">
+        <v>2023-04-01</v>
+      </c>
+      <c r="L2" t="str">
+        <v>2026-02-12</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>startup-vaultedge</v>
+      </c>
+      <c r="B3" t="str">
+        <v>VaultEdge</v>
+      </c>
+      <c r="C3" t="str">
+        <v>PRIVATE</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
         <v>25000</v>
       </c>
-      <c r="K2" t="str">
-        <v>2025-08-01</v>
-      </c>
-      <c r="L2" t="str">
+      <c r="F3">
+        <v>25000</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Pre-seed. Decentralized identity for fintech. Earliest stage, highest risk.</v>
+      </c>
+      <c r="H3" t="str">
+        <v>taxable</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Direct Investment</v>
+      </c>
+      <c r="J3">
+        <v>25000</v>
+      </c>
+      <c r="K3" t="str">
+        <v>2025-06-01</v>
+      </c>
+      <c r="L3" t="str">
         <v>2026-02-12</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>